<commit_message>
1. spring-rest-handson HOL DONE
</commit_message>
<xml_diff>
--- a/[Solve Tracking] DN - Java FSE Mandatory hands-on detail.xlsx
+++ b/[Solve Tracking] DN - Java FSE Mandatory hands-on detail.xlsx
@@ -1069,13 +1069,13 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="8" t="s">
         <v>51</v>
       </c>
       <c r="D25" s="9" t="s">
@@ -1086,13 +1086,13 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="8" t="s">
         <v>54</v>
       </c>
       <c r="D26" s="9"/>

</xml_diff>

<commit_message>
5. JWT-handson HOL done / check [Solve Tracking] DN - Java FSE Mandatory hands-on detail
</commit_message>
<xml_diff>
--- a/[Solve Tracking] DN - Java FSE Mandatory hands-on detail.xlsx
+++ b/[Solve Tracking] DN - Java FSE Mandatory hands-on detail.xlsx
@@ -1099,52 +1099,52 @@
       <c r="E26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="8" t="s">
         <v>56</v>
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="8" t="s">
         <v>57</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="8" t="s">
         <v>58</v>
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="8" t="s">
         <v>60</v>
       </c>
       <c r="D30" s="9"/>

</xml_diff>

<commit_message>
JUnit HOL Done All
</commit_message>
<xml_diff>
--- a/[Solve Tracking] DN - Java FSE Mandatory hands-on detail.xlsx
+++ b/[Solve Tracking] DN - Java FSE Mandatory hands-on detail.xlsx
@@ -347,7 +347,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -370,6 +370,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF6F9D4"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF6F9D4"/>
       </patternFill>
     </fill>
   </fills>
@@ -428,7 +434,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -465,7 +471,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -786,8 +804,8 @@
       <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
@@ -799,8 +817,8 @@
       <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
@@ -812,8 +830,8 @@
       <c r="C5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
@@ -825,8 +843,8 @@
       <c r="C6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
@@ -838,8 +856,8 @@
       <c r="C7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
@@ -851,95 +869,95 @@
       <c r="C8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="10"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="8"/>
       <c r="C12" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
@@ -1082,10 +1100,10 @@
       <c r="C25" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1099,8 +1117,8 @@
       <c r="C26" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
@@ -1112,8 +1130,8 @@
       <c r="C27" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
@@ -1125,8 +1143,8 @@
       <c r="C28" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
@@ -1138,8 +1156,8 @@
       <c r="C29" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
@@ -1151,32 +1169,32 @@
       <c r="C30" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="E31" s="11" t="s">
+      <c r="E31" s="14" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="12" t="s">
+      <c r="A32" s="10"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="15" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1284,10 +1302,10 @@
       <c r="C39" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E39" s="7" t="s">
+      <c r="E39" s="9" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1301,10 +1319,10 @@
       <c r="C40" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E40" s="7" t="s">
+      <c r="E40" s="9" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1318,10 +1336,10 @@
       <c r="C41" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="E41" s="7" t="s">
+      <c r="E41" s="9" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1335,90 +1353,90 @@
       <c r="C42" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="9" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="9" t="s">
+      <c r="A43" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B43" s="10" t="s">
+      <c r="B43" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="C43" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
+      <c r="C43" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="9" t="s">
+      <c r="A44" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="B44" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="C44" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D44" s="9"/>
+      <c r="C44" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D44" s="10"/>
       <c r="E44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="9" t="s">
+      <c r="A45" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B45" s="10" t="s">
+      <c r="B45" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="C45" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
+      <c r="C45" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="9" t="s">
+      <c r="A46" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B46" s="10" t="s">
+      <c r="B46" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
+      <c r="C46" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="9" t="s">
+      <c r="A47" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B47" s="10" t="s">
+      <c r="B47" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="C47" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
+      <c r="C47" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B48" s="13" t="s">
+      <c r="B48" s="16" t="s">
         <v>92</v>
       </c>
       <c r="C48" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>